<commit_message>
Refresh KO research note + model (Q2 FY2026, HOLD)
</commit_message>
<xml_diff>
--- a/assets/files/coca-cola-business-model.xlsx
+++ b/assets/files/coca-cola-business-model.xlsx
@@ -1376,7 +1376,7 @@
     <row r="2">
       <c r="A2" s="58" t="inlineStr">
         <is>
-          <t>USD; per-share USD. Dividend aristocrat (63+ yrs) — DDM-led. Live $82 (Jul 2026), 4,310M shares, net debt ~$29bn.</t>
+          <t>USD; per-share USD. Dividend King (64 yrs) — DDM-led valuation. Live $87 (28-Jul-2026), post-Q2 record high.</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B5" s="141" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6">
@@ -1434,7 +1434,7 @@
         </is>
       </c>
       <c r="B9" s="58" t="n">
-        <v>3.15</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="10">
@@ -1454,7 +1454,7 @@
         </is>
       </c>
       <c r="B11" s="141" t="n">
-        <v>15100</v>
+        <v>15300</v>
       </c>
     </row>
     <row r="12">
@@ -1633,7 +1633,7 @@
     <row r="25">
       <c r="A25" s="58" t="inlineStr">
         <is>
-          <t>Upside / (downside) vs $82</t>
+          <t>Upside / (downside) vs price</t>
         </is>
       </c>
       <c r="B25" s="144">
@@ -4951,10 +4951,8 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="B4" s="124" t="inlineStr">
-        <is>
-          <t>Price ($)</t>
-        </is>
+      <c r="B4" s="124" t="n">
+        <v>87</v>
       </c>
       <c r="C4" s="124" t="inlineStr">
         <is>

</xml_diff>